<commit_message>
Aktueller Stand, Produktivtest steht bevor
</commit_message>
<xml_diff>
--- a/UPL_Performer/Data/Config.xlsx
+++ b/UPL_Performer/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\timotheus.vrettos\develop\develop_RPA\uipath-rpa_upl\UPL_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA06DEF3-B123-46AB-80E7-D7A9CDF9A801}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B41AF603-F93F-43B8-A44C-E99F7979E445}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="87">
   <si>
     <t>Name</t>
   </si>
@@ -281,13 +281,31 @@
   </si>
   <si>
     <t>msedge, EXCEL</t>
+  </si>
+  <si>
+    <t>rpa009_Webex_Token</t>
+  </si>
+  <si>
+    <t>58921f80-2dc3-11f1-adea-27022ecb5c33</t>
+  </si>
+  <si>
+    <t>WebexRoomID</t>
+  </si>
+  <si>
+    <t>https://webexapis.com/v1/messages</t>
+  </si>
+  <si>
+    <t>WebexApiUrl</t>
+  </si>
+  <si>
+    <t>rpa009_DimaLink</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -311,6 +329,19 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -329,10 +360,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -344,8 +376,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Link" xfId="1" builtinId="8"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -752,9 +791,30 @@
         <v>70</v>
       </c>
     </row>
-    <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
+    <row r="9" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A9" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A10" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A11" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="13" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="14" spans="1:26" ht="14.25" customHeight="1"/>
@@ -1744,8 +1804,11 @@
     <row r="998" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
+  <hyperlinks>
+    <hyperlink ref="B10" r:id="rId1" xr:uid="{603F44BE-C244-41D2-AE20-6390D102C87B}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -3105,8 +3168,12 @@
       </c>
     </row>
     <row r="5" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A5" s="6"/>
-      <c r="B5" s="6"/>
+      <c r="A5" t="s">
+        <v>86</v>
+      </c>
+      <c r="B5" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="7" spans="1:26" ht="14.25" customHeight="1"/>
@@ -4105,5 +4172,6 @@
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Webex Token angepasst & Fehlerprotokoll hinzugefügt
</commit_message>
<xml_diff>
--- a/UPL_Performer/Data/Config.xlsx
+++ b/UPL_Performer/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\timotheus.vrettos\develop\develop_RPA\uipath-rpa_upl\UPL_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EBD3000-9D42-4C65-835F-5EF249A5B049}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B96DE53-1F5A-4471-8BAE-544D473DCE68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-8460" yWindow="-14235" windowWidth="21600" windowHeight="11235" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -265,9 +265,6 @@
     <t>02 Wassertemperatur.csv</t>
   </si>
   <si>
-    <t>rpa009_Webex_Token</t>
-  </si>
-  <si>
     <t>58921f80-2dc3-11f1-adea-27022ecb5c33</t>
   </si>
   <si>
@@ -284,6 +281,9 @@
   </si>
   <si>
     <t>msedge, EXCEL, wfica32</t>
+  </si>
+  <si>
+    <t>global_WebEx_Token</t>
   </si>
 </sst>
 </file>
@@ -778,26 +778,26 @@
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
@@ -1880,7 +1880,7 @@
         <v>45</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>46</v>
@@ -3122,10 +3122,10 @@
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1">
       <c r="A3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>

<commit_message>
Export aufteilen & Konsolidieren. Webex auf Prod/Test Room geteilt
</commit_message>
<xml_diff>
--- a/UPL_Performer/Data/Config.xlsx
+++ b/UPL_Performer/Data/Config.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\timotheus.vrettos\develop\develop_RPA\uipath-rpa_upl\UPL_Performer\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B96DE53-1F5A-4471-8BAE-544D473DCE68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1981678E-F49A-481D-9ACE-EDD6CE541DC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="81">
   <si>
     <t>Name</t>
   </si>
@@ -265,12 +265,6 @@
     <t>02 Wassertemperatur.csv</t>
   </si>
   <si>
-    <t>58921f80-2dc3-11f1-adea-27022ecb5c33</t>
-  </si>
-  <si>
-    <t>WebexRoomID</t>
-  </si>
-  <si>
     <t>https://webexapis.com/v1/messages</t>
   </si>
   <si>
@@ -284,13 +278,16 @@
   </si>
   <si>
     <t>global_WebEx_Token</t>
+  </si>
+  <si>
+    <t>rpa009_Webex_RoomID</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -312,12 +309,6 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Segoe UI"/>
       <family val="2"/>
     </font>
     <font>
@@ -347,9 +338,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
@@ -361,10 +352,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -682,7 +670,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z998"/>
+  <dimension ref="A1:Z997"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.44140625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="43.5546875" customWidth="1"/>
@@ -786,18 +774,18 @@
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>77</v>
+        <v>79</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A11" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>81</v>
+      <c r="A11" t="s">
+        <v>80</v>
+      </c>
+      <c r="B11" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1"/>
@@ -1786,11 +1774,10 @@
     <row r="995" ht="14.25" customHeight="1"/>
     <row r="996" ht="14.25" customHeight="1"/>
     <row r="997" ht="14.25" customHeight="1"/>
-    <row r="998" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="2"/>
   <hyperlinks>
-    <hyperlink ref="B10" r:id="rId1" xr:uid="{603F44BE-C244-41D2-AE20-6390D102C87B}"/>
+    <hyperlink ref="B9" r:id="rId1" xr:uid="{603F44BE-C244-41D2-AE20-6390D102C87B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
@@ -1880,7 +1867,7 @@
         <v>45</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>46</v>
@@ -3122,10 +3109,10 @@
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1">
       <c r="A3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1"/>

</xml_diff>